<commit_message>
Mejora de formato y validacion del reporte
</commit_message>
<xml_diff>
--- a/output/reporte_final.xlsx
+++ b/output/reporte_final.xlsx
@@ -18,14 +18,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -48,8 +53,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,34 +424,42 @@
   </sheetPr>
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>producto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>cantidad</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ciudad</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>archivo_origen</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>total</t>
         </is>
@@ -472,7 +487,7 @@
           <t>ventas_enero.xlsx</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="2" t="n">
         <v>1600</v>
       </c>
     </row>
@@ -498,7 +513,7 @@
           <t>ventas_enero.xlsx</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="2" t="n">
         <v>100</v>
       </c>
     </row>
@@ -524,7 +539,7 @@
           <t>ventas_enero.xlsx</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="2" t="n">
         <v>135</v>
       </c>
     </row>
@@ -550,7 +565,7 @@
           <t>ventas_febrero.xlsx</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="2" t="n">
         <v>800</v>
       </c>
     </row>
@@ -576,7 +591,7 @@
           <t>ventas_febrero.xlsx</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="2" t="n">
         <v>40</v>
       </c>
     </row>
@@ -602,7 +617,7 @@
           <t>ventas_febrero.xlsx</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="2" t="n">
         <v>45</v>
       </c>
     </row>
@@ -628,7 +643,7 @@
           <t>ventas_marzo.xlsx</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="2" t="n">
         <v>3200</v>
       </c>
     </row>
@@ -654,7 +669,7 @@
           <t>ventas_marzo.xlsx</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="2" t="n">
         <v>200</v>
       </c>
     </row>
@@ -680,7 +695,7 @@
           <t>ventas_marzo.xlsx</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="2" t="n">
         <v>90</v>
       </c>
     </row>
@@ -697,14 +712,18 @@
   </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ciudad</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>total</t>
         </is>
@@ -713,11 +732,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Arecibo</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>270</v>
+          <t>San Juan</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>5600</v>
       </c>
     </row>
     <row r="3">
@@ -726,18 +745,18 @@
           <t>Ponce</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>340</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>San Juan</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>5600</v>
+          <t>Arecibo</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -753,14 +772,18 @@
   </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>producto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>total</t>
         </is>
@@ -772,7 +795,7 @@
           <t>laptop</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>5600</v>
       </c>
     </row>
@@ -782,7 +805,7 @@
           <t>mouse</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>340</v>
       </c>
     </row>
@@ -792,7 +815,7 @@
           <t>teclado</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>270</v>
       </c>
     </row>

</xml_diff>